<commit_message>
feat(F-NAR-019): ATOM-AUT.ROU.001-01 Le train de l'allée
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.ROU.001-01.xlsx
+++ b/stories/arbres/ATOM-AUT.ROU.001-01.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>maison du village, chambre puis jardin, le matin</t>
+          <t>maison du village, chambre puis jardin, allée des dalles, le matin</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Chouchou veut faire rouler son train sur l'allée. Elle prend tout à la fois, une roue part. Une chose puis la suivante, le wagon avance sur les dalles tièdes.</t>
+          <t>L'odeur du linge arrive avant le soleil. Sur le toit rouge, un éclat de wagon brille. Chouchou veut la dernière dalle, maintenant. Elle prend train et chaussure : une roue part. Elle pousse trop fort : le wagon tombe sur le flanc. Elle refuse de foncer, remet la roue, pose le train. Une feuille barre la dalle ; elle écarte, le wagon avance. Près du portail, l'éclat de wagon tient sur le toit.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Sur le rebord, un petit train de bois attend. Le toit du wagon est rouge, un peu pâle. Une roue brille encore, toute ronde. La nuit vient juste de partir. Le jardin sent la terre mouillée. Les dalles de l'allée sont fraîches. Une goutte tombe d'une feuille. Un merle chante tout au fond. Dans la maison, le couloir sent le linge. Chouchou, tu vois ton train ? Oui, papa. Il veut l'allée. L'allée est encore un peu froide. En ce moment, Chouchou est dans son lit. La couverture est chaude, un peu lourde. Elle sent le savon de la lessive. Je sors le train. Chouchou prend le wagon d'une main. De l'autre, elle attrape une chaussure. Le wagon bascule. Une petite roue part sous la chaise. Oh. La roue. Le train a besoin de toi, toute entière. Une chose, puis la suivante. Chouchou pose la chaussure près du lit. Elle cherche la roue du bout des doigts. Le bois est lisse, un peu frais. Je l'ai. D'abord on se lève. Chouchou pousse la couverture. Ses pieds trouvent le tapis beige. Le tapis est doux sous les orteils. Tu es debout ? Oui, maman. Ensuite le pull, pour conduire.</t>
+          <t>L'odeur du linge arrive dans la chambre, avant le soleil. Un carré de buée s'ouvre sur la vitre. Sur le rebord, le train de bois attend. Le toit du wagon est rouge, un peu pâle. Sur le rouge, un éclat de wagon brille. Il est petit, papa. C'est le soleil sur le bois. Le rebord tient le train comme une petite gare. Le rouge du toit chauffe un peu, sous la buée. Le jardin sent la terre mouillée. Les dalles de l'allée sont fraîches. Une goutte tombe d'une feuille. Dans la maison, le couloir sent le linge. La nuit vient de partir. Il veut l'allée, maintenant ! Jusqu'où, Chouchou ? Jusqu'à la dernière dalle ! La couverture est chaude, un peu lourde. Elle sent le savon de la lessive. Chouchou, tu vois ton train ? Oui, papa. Le pull bleu repose sur la chaise. En ce moment, Chouchou saisit le train. Le bois est lisse, un peu frais. De l'autre main, elle attrape une chaussure. Le wagon bascule. Une petite roue part sous la chaise. Oh. La roue. Chouchou pousse la couverture. Ses pieds trouvent le tapis beige. Tu es debout ? Oui, maman. Je le pousse, vite ! Elle pose le train sur le tapis beige. Le tapis est doux sous les orteils. Elle pousse trop fort, d'un coup. Le wagon glisse, puis tombe sur le flanc. Les roues tournent dans le vide. Ça ne veut pas, papa. Le sourire de Chouchou disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Tu regardes sous la chaise ?</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Sur le rebord, un petit train de bois attend. Le toit du wagon est rouge, un peu pâle. Une roue brille encore, toute ronde. La nuit vient juste de partir. Le jardin sent la terre mouillée. Les dalles de l'allée sont fraîches. Une goutte tombe d'une feuille. Un merle chante tout au fond. Dans la maison, le couloir sent le linge. Chouchou, tu vois ton train ? Oui, papa. Il veut l'allée. L'allée est encore un peu froide. En ce moment, Chouchou est dans son lit. La couverture est chaude, un peu lourde. Elle sent le savon de la lessive. Je sors le train. Chouchou prend le wagon d'une main. De l'autre, elle attrape une chaussure. Le wagon bascule. Une petite roue part sous la chaise. Oh. La roue. Le train a besoin de toi, toute entière. Une chose, puis la suivante. Chouchou pose la chaussure près du lit. Elle cherche la roue du bout des doigts. Le bois est lisse, un peu frais. Je l'ai. D'abord on se lève. Chouchou pousse la couverture. Ses pieds trouvent le tapis beige. Le tapis est doux sous les orteils. Tu es debout ? Oui, maman. Ensuite le pull, pour conduire.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;L'odeur du linge arrive dans la chambre, avant le soleil. Un carré de buée s'ouvre sur la vitre. Sur le rebord, le train de bois attend. Le toit du wagon est rouge, un peu pâle. Sur le rouge, un &lt;emphasis level="moderate"&gt;éclat de wagon&lt;/emphasis&gt; brille. Il est petit, papa. C'est le soleil sur le bois. Le rebord tient le train comme une petite gare. Le rouge du toit chauffe un peu, sous la buée. Le jardin sent la terre mouillée. Les dalles de l'allée sont fraîches. Une goutte tombe d'une feuille. Dans la maison, le couloir sent le linge. La nuit vient de partir. Il veut l'allée, maintenant ! Jusqu'où, Chouchou ? Jusqu'à la dernière dalle ! La couverture est chaude, un peu lourde. Elle sent le savon de la lessive. Chouchou, tu vois ton train ? Oui, papa. Le pull bleu repose sur la chaise. En ce moment, Chouchou saisit le train. Le bois est lisse, un peu frais. De l'autre main, elle attrape une chaussure. Le wagon bascule. Une petite roue part sous la chaise. Oh. La roue. Chouchou pousse la couverture. Ses pieds trouvent le tapis beige. Tu es debout ? Oui, maman. Je le pousse, vite ! Elle pose le train sur le tapis beige. Le tapis est doux sous les orteils. Elle pousse trop fort, d'un coup. Le wagon glisse, puis tombe sur le flanc. Les roues tournent dans le vide. Ça ne veut pas, papa. Le sourire de Chouchou disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Tu regardes sous la chaise ?&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Le soleil entre dans la chambre. Hugo ouvre les yeux. Le drap est chaud. Papa dit : c'est le matin. &lt;emphasis&gt;une&lt;/emphasis&gt; étape après l'autre. D'abord, Hugo se lève. Ses pieds touchent le tapis. Le tapis est doux. Ensuite, Hugo s'habille. Il met le pull bleu. Il met le pantalon. Les chaussettes aussi. Maman dit : maintenant, le déjeuner. Hugo s'assoit à table. Il mange du pain. Il boit du lait tiède. Papa dit : ensuite, le sac. Hugo met la gourde dans le sac. Hugo met le doudou dans le sac. Chaque étape est finie, alors Hugo est prêt. Papa dit : une étape après l'autre, et c'est plus calme. [pause]</t>
+          <t>L'odeur du linge arrive dans la chambre, avant le soleil. Un carré de buée s'ouvre sur la vitre. Sur le rebord, le train de bois attend. Le toit du wagon est rouge, un peu pâle. Sur le rouge, un &lt;emphasis&gt;éclat de wagon&lt;/emphasis&gt; brille. Il est petit, papa. C'est le soleil sur le bois. Le rebord tient le train comme une petite gare. Le rouge du toit chauffe un peu, sous la buée. Le jardin sent la terre mouillée. Les dalles de l'allée sont fraîches. Une goutte tombe d'une feuille. Dans la maison, le couloir sent le linge. La nuit vient de partir. Il veut l'allée, maintenant ! Jusqu'où, Chouchou ? Jusqu'à la dernière dalle ! La couverture est chaude, un peu lourde. Elle sent le savon de la lessive. Chouchou, tu vois ton train ? Oui, papa. Le pull bleu repose sur la chaise. En ce moment, Chouchou saisit le train. Le bois est lisse, un peu frais. De l'autre main, elle attrape une chaussure. Le wagon bascule. Une petite roue part sous la chaise. Oh. La roue. Chouchou pousse la couverture. Ses pieds trouvent le tapis beige. Tu es debout ? Oui, maman. Je le pousse, vite ! Elle pose le train sur le tapis beige. Le tapis est doux sous les orteils. Elle pousse trop fort, d'un coup. Le wagon glisse, puis tombe sur le flanc. Les roues tournent dans le vide. Ça ne veut pas, papa. Le sourire de Chouchou disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa se baisse à sa hauteur. Tu regardes sous la chaise ? [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>une</t>
+          <t>éclat de wagon</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,50 +1321,63 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_la_derniere_dalle_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Sur le rebord, un petit train de bois attend.
+          <t>narrateur|L'odeur du linge arrive dans la chambre, avant le soleil.
+narrateur|Un carré de buée s'ouvre sur la vitre.
+narrateur|Sur le rebord, le train de bois attend.
 narrateur|Le toit du wagon est rouge, un peu pâle.
-narrateur|Une roue brille encore, toute ronde.
-narrateur|La nuit vient juste de partir.
+narrateur|Sur le rouge, un éclat de wagon brille.
+enfant-f|Il est petit, papa.
+papa|C'est le soleil sur le bois.
+narrateur|Le rebord tient le train comme une petite gare.
+narrateur|Le rouge du toit chauffe un peu, sous la buée.
 narrateur|Le jardin sent la terre mouillée.
 narrateur|Les dalles de l'allée sont fraîches.
 narrateur|Une goutte tombe d'une feuille.
-narrateur|Un merle chante tout au fond.
 narrateur|Dans la maison, le couloir sent le linge.
+narrateur|La nuit vient de partir.
+enfant-f|Il veut l'allée, maintenant !
+maman|Jusqu'où, Chouchou ?
+enfant-f|Jusqu'à la dernière dalle !
+narrateur|La couverture est chaude, un peu lourde.
+narrateur|Elle sent le savon de la lessive.
 papa|Chouchou, tu vois ton train ?
 enfant-f|Oui, papa.
-enfant-f|Il veut l'allée.
-maman|L'allée est encore un peu froide.
-narrateur|En ce moment, Chouchou est dans son lit.
-narrateur|La couverture est chaude, un peu lourde.
-narrateur|Elle sent le savon de la lessive.
-enfant-f|Je sors le train.
-narrateur|Chouchou prend le wagon d'une main.
-narrateur|De l'autre, elle attrape une chaussure.
+narrateur|Le pull bleu repose sur la chaise.
+narrateur|En ce moment, Chouchou saisit le train.
+narrateur|Le bois est lisse, un peu frais.
+narrateur|De l'autre main, elle attrape une chaussure.
 narrateur|Le wagon bascule.
 narrateur|Une petite roue part sous la chaise.
 enfant-f|Oh.
 enfant-f|La roue.
-papa|Le train a besoin de toi, toute entière.
-maman|Une chose, puis la suivante.
-narrateur|Chouchou pose la chaussure près du lit.
-narrateur|Elle cherche la roue du bout des doigts.
-narrateur|Le bois est lisse, un peu frais.
-enfant-f|Je l'ai.
-papa|D'abord on se lève.
 narrateur|Chouchou pousse la couverture.
 narrateur|Ses pieds trouvent le tapis beige.
-narrateur|Le tapis est doux sous les orteils.
 maman|Tu es debout ?
 enfant-f|Oui, maman.
-papa|Ensuite le pull, pour conduire.</t>
+enfant-f|Je le pousse, vite !
+narrateur|Elle pose le train sur le tapis beige.
+narrateur|Le tapis est doux sous les orteils.
+narrateur|Elle pousse trop fort, d'un coup.
+narrateur|Le wagon glisse, puis tombe sur le flanc.
+narrateur|Les roues tournent dans le vide.
+enfant-f|Ça ne veut pas, papa.
+narrateur|Le sourire de Chouchou disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa se baisse à sa hauteur.
+papa|Tu regardes sous la chaise ?</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>reveil</t>
+          <t>reveil,train</t>
         </is>
       </c>
     </row>
@@ -1391,27 +1404,27 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Chouchou veut l'allée. Comment se prépare-t-elle ?</t>
+          <t>Chouchou veut la dernière dalle. Comment le wagon avance-t-il ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Chouchou veut l'allée. Comment se prépare-t-elle ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Chouchou veut la dernière dalle. Comment le &lt;emphasis level="moderate"&gt;wagon&lt;/emphasis&gt; avance-t-il ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Hugo se prépare. Comment avance-t-il ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Chouchou veut la dernière dalle. Comment le &lt;emphasis&gt;wagon&lt;/emphasis&gt; avance-t-il ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>une chose</t>
+          <t>il roule</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>une chose | puis l'autre | d'abord | doucement | une chose puis l'autre | puis la suivante</t>
+          <t>il roule | roule | avec les roues | sur les dalles | les roues | le wagon roule</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -1426,7 +1439,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Elle fait une chose, puis la suivante. Comment se prépare Chouchou ?</t>
+          <t>Le wagon est tombé sur le flanc. Comment avance-t-il ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1464,7 +1477,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1475,7 +1488,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1490,34 +1503,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>wagon</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1532,23 +1549,23 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=le_wagon_avance_quand_les_roues_touchent; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Chouchou veut l'allée.
-narrateur|Comment se prépare-t-elle ?</t>
+          <t>narrateur|Chouchou veut la dernière dalle.
+narrateur|Comment le wagon avance-t-il ?</t>
         </is>
       </c>
     </row>
@@ -1575,17 +1592,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Chouchou a la petite roue dans la main. Une chose, puis la suivante. Maintenant, le pull du train. Le pull bleu est sur la chaise. Les manches sont un peu longues. Chouchou enfile le pull. Je relève une manche. Je peux conduire. Oui. Ensuite, on va à table. La cuisine sent le lait tiède. La fenêtre est un peu embuée. Chouchou s'assoit. Ses pieds touchent le carrelage frais. Tu veux le bol bleu ? Oui, le bleu. Elle mange un bout de pain. La croûte fait un petit bruit. C'est la gare, ici. Le train attend. Il attend dans le sac. Merci, Chouchou.</t>
+          <t>Chouchou laisse la chaussure près du lit. Elle pose un genou sur le tapis. Sa main passe sous la chaise. Le bois de la roue est lisse, un peu frais. Je l'ai. Elle remet la petite roue. Toc. Le wagon se tient droit. Tu peux partir. Tes chaussures, Chouchou ? Oui, maman. Elle pose une chaussure, puis l'autre. Les lacets font un petit bruit. On ouvre ? L'allée. Maman ouvre la porte. L'air sent la terre mouillée. Les dalles commencent à être tièdes. Chouchou pose le train sur une dalle sèche. Vite, jusqu'au bout ! Elle pousse trop fort. Le wagon penche, puis se couche. Oh. Elle ne reprend pas trop vite. Une goutte tombe, loin, sur une dalle. Elle écoute l'allée, un instant. Sur le toit, l'éclat de wagon brille. Il est là. Chouchou refuse de foncer. Elle redresse le wagon, lentement. Elle donne une petite poussée. Le wagon avance. Toc. Le bois frotte la pierre. Ça fait un petit bruit. Une autre dalle, plus loin. Il roule ! Merci, Chouchou. Il va tout seul. Tu le vois, toi ? Oui, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Chouchou a la petite roue dans la main. Une chose, puis la suivante. Maintenant, le pull du train. Le pull bleu est sur la chaise. Les manches sont un peu longues. Chouchou enfile le pull. Je relève une manche. Je peux conduire. Oui. Ensuite, on va à table. La cuisine sent le lait tiède. La fenêtre est un peu embuée. Chouchou s'assoit. Ses pieds touchent le carrelage frais. Tu veux le bol bleu ? Oui, le bleu. Elle mange un bout de pain. La croûte fait un petit bruit. C'est la gare, ici. Le train attend. Il attend dans le sac. Merci, Chouchou.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Chouchou laisse la chaussure près du lit. Elle pose un genou sur le tapis. Sa main passe sous la chaise. Le bois de la roue est lisse, un peu frais. Je l'ai. Elle remet la petite roue. Toc. Le wagon se tient droit. Tu peux partir. Tes chaussures, Chouchou ? Oui, maman. Elle pose une chaussure, puis l'autre. Les lacets font un petit bruit. On ouvre ? L'allée. Maman ouvre la porte. L'air sent la terre mouillée. Les &lt;emphasis level="moderate"&gt;dalle&lt;/emphasis&gt;s commencent à être tièdes. Chouchou pose le train sur une dalle sèche. Vite, jusqu'au bout ! Elle pousse trop fort. Le wagon penche, puis se couche. Oh. Elle ne reprend pas trop vite. Une goutte tombe, loin, sur une dalle. Elle écoute l'allée, un instant. Sur le toit, l'éclat de wagon brille. Il est là. Chouchou refuse de foncer. Elle redresse le wagon, lentement. Elle donne une petite poussée. Le wagon avance. Toc. Le bois frotte la pierre. Ça fait un petit bruit. Une autre dalle, plus loin. Il roule ! Merci, Chouchou. Il va tout seul. Tu le vois, toi ? Oui, maman.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Hugo a fait l'étape dite. Se lever. S'habiller. Déje&lt;emphasis&gt;une&lt;/emphasis&gt;r. Le sac. Une étape après l'autre. [pause]</t>
+          <t>Chouchou laisse la chaussure près du lit. Elle pose un genou sur le tapis. Sa main passe sous la chaise. Le bois de la roue est lisse, un peu frais. Je l'ai. Elle remet la petite roue. Toc. Le wagon se tient droit. Tu peux partir. Tes chaussures, Chouchou ? Oui, maman. Elle pose une chaussure, puis l'autre. Les lacets font un petit bruit. On ouvre ? L'allée. Maman ouvre la porte. L'air sent la terre mouillée. Les &lt;emphasis&gt;dalle&lt;/emphasis&gt;s commencent à être tièdes. Chouchou pose le train sur une dalle sèche. Vite, jusqu'au bout ! Elle pousse trop fort. Le wagon penche, puis se couche. Oh. Elle ne reprend pas trop vite. Une goutte tombe, loin, sur une dalle. Elle écoute l'allée, un instant. Sur le toit, l'éclat de wagon brille. Il est là. Chouchou refuse de foncer. Elle redresse le wagon, lentement. Elle donne une petite poussée. Le wagon avance. Toc. Le bois frotte la pierre. Ça fait un petit bruit. Une autre dalle, plus loin. Il roule ! Merci, Chouchou. Il va tout seul. Tu le vois, toi ? Oui, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1632,7 +1649,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1640,10 +1657,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1666,30 +1683,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>une</t>
+          <t>dalle</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1698,10 +1715,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1714,33 +1731,57 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=concentration puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_pose_le_train_sans_foncer; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Chouchou a la petite roue dans la main.
-maman|Une chose, puis la suivante.
-papa|Maintenant, le pull du train.
-narrateur|Le pull bleu est sur la chaise.
-narrateur|Les manches sont un peu longues.
-narrateur|Chouchou enfile le pull.
-papa|Je relève une manche.
-enfant-f|Je peux conduire.
-maman|Oui.
-maman|Ensuite, on va à table.
-narrateur|La cuisine sent le lait tiède.
-narrateur|La fenêtre est un peu embuée.
-narrateur|Chouchou s'assoit.
-narrateur|Ses pieds touchent le carrelage frais.
-maman|Tu veux le bol bleu ?
-enfant-f|Oui, le bleu.
-narrateur|Elle mange un bout de pain.
-narrateur|La croûte fait un petit bruit.
-papa|C'est la gare, ici.
-enfant-f|Le train attend.
-maman|Il attend dans le sac.
-papa|Merci, Chouchou.</t>
+          <t>narrateur|Chouchou laisse la chaussure près du lit.
+narrateur|Elle pose un genou sur le tapis.
+narrateur|Sa main passe sous la chaise.
+narrateur|Le bois de la roue est lisse, un peu frais.
+enfant-f|Je l'ai.
+narrateur|Elle remet la petite roue.
+narrateur|Toc.
+narrateur|Le wagon se tient droit.
+enfant-f|Tu peux partir.
+maman|Tes chaussures, Chouchou ?
+enfant-f|Oui, maman.
+narrateur|Elle pose une chaussure, puis l'autre.
+narrateur|Les lacets font un petit bruit.
+papa|On ouvre ?
+enfant-f|L'allée.
+narrateur|Maman ouvre la porte.
+narrateur|L'air sent la terre mouillée.
+narrateur|Les dalles commencent à être tièdes.
+narrateur|Chouchou pose le train sur une dalle sèche.
+enfant-f|Vite, jusqu'au bout !
+narrateur|Elle pousse trop fort.
+narrateur|Le wagon penche, puis se couche.
+enfant-f|Oh.
+narrateur|Elle ne reprend pas trop vite.
+narrateur|Une goutte tombe, loin, sur une dalle.
+narrateur|Elle écoute l'allée, un instant.
+narrateur|Sur le toit, l'éclat de wagon brille.
+enfant-f|Il est là.
+narrateur|Chouchou refuse de foncer.
+narrateur|Elle redresse le wagon, lentement.
+narrateur|Elle donne une petite poussée.
+narrateur|Le wagon avance.
+narrateur|Toc.
+narrateur|Le bois frotte la pierre.
+narrateur|Ça fait un petit bruit.
+narrateur|Une autre dalle, plus loin.
+enfant-f|Il roule !
+papa|Merci, Chouchou.
+enfant-f|Il va tout seul.
+maman|Tu le vois, toi ?
+enfant-f|Oui, maman.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>roue,dalles</t>
         </is>
       </c>
     </row>
@@ -1767,17 +1808,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Le sac, maintenant. Le sac bleu est près de la porte. Chouchou pose le wagon dedans. Elle remet la petite roue. Ça fait toc, tout doux. Tu as mis le train ? Oui, maman. Chouchou met ses chaussures. Les lacets font un petit bruit. On ouvre ? L'allée. Maman ouvre la porte. L'air sent la terre mouillée. Les dalles commencent à être tièdes. Chouchou sort le train. Elle le pose sur une dalle. Roule. Le wagon avance. Toc. Une autre dalle, plus loin. Il va jusqu'au merle. Une chose, puis la suivante. Et le train est parti. Le merle penche la tête. Il me regarde.</t>
+          <t>Il va jusqu'à la dernière dalle ? Oui, papa. Une feuille mouillée barre une dalle. Le wagon s'arrête contre le bord. Je le porte ! Elle saisit le train trop vite. Une roue quitte la dalle. Oh. Chouchou s'arrête. Ses mains se ferment, puis s'ouvrent. Elle refuse de foncer. Le train revient sur la dalle sèche. Elle écarte la feuille du bout des doigts. La dalle est libre, un peu sombre. Roule. Le wagon avance. Toc. Une autre dalle, plus loin. L'éclat de wagon tremble, puis tient. Il a passé la feuille. La dernière dalle est près du portail. J'y vais. Chouchou marche à côté, sans le porter. Le bois continue son petit bruit.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Le sac, maintenant. Le sac bleu est près de la porte. Chouchou pose le wagon dedans. Elle remet la petite roue. Ça fait toc, tout doux. Tu as mis le train ? Oui, maman. Chouchou met ses chaussures. Les lacets font un petit bruit. On ouvre ? L'allée. Maman ouvre la porte. L'air sent la terre mouillée. Les dalles commencent à être tièdes. Chouchou sort le train. Elle le pose sur une dalle. Roule. Le wagon avance. Toc. Une autre dalle, plus loin. Il va jusqu'au merle. Une chose, puis la suivante. Et le train est parti. Le merle penche la tête. Il me regarde.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Il va jusqu'à la dernière dalle ? Oui, papa. Une &lt;emphasis level="moderate"&gt;feuille&lt;/emphasis&gt; mouillée barre une dalle. Le wagon s'arrête contre le bord. Je le porte ! Elle saisit le train trop vite. Une roue quitte la dalle. Oh. Chouchou s'arrête. Ses mains se ferment, puis s'ouvrent. Elle refuse de foncer. Le train revient sur la dalle sèche. Elle écarte la feuille du bout des doigts. La dalle est libre, un peu sombre. Roule. Le wagon avance. Toc. Une autre dalle, plus loin. L'éclat de wagon tremble, puis tient. Il a passé la feuille. La dernière dalle est près du portail. J'y vais. Chouchou marche à côté, sans le porter. Le bois continue son petit bruit.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Hugo met les chaussures. Maman ouvre la porte. L'air sent le matin. [pause]</t>
+          <t>Il va jusqu'à la dernière dalle ? Oui, papa. Une &lt;emphasis&gt;feuille&lt;/emphasis&gt; mouillée barre une dalle. Le wagon s'arrête contre le bord. Je le porte ! Elle saisit le train trop vite. Une roue quitte la dalle. Oh. Chouchou s'arrête. Ses mains se ferment, puis s'ouvrent. Elle refuse de foncer. Le train revient sur la dalle sèche. Elle écarte la feuille du bout des doigts. La dalle est libre, un peu sombre. Roule. Le wagon avance. Toc. Une autre dalle, plus loin. L'éclat de wagon tremble, puis tient. Il a passé la feuille. La dernière dalle est près du portail. J'y vais. Chouchou marche à côté, sans le porter. Le bois continue son petit bruit. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1824,7 +1865,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1832,10 +1873,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1856,28 +1897,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>feuille</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1886,10 +1931,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1900,39 +1945,42 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_porter_le_train; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>papa|Le sac, maintenant.
-narrateur|Le sac bleu est près de la porte.
-narrateur|Chouchou pose le wagon dedans.
-narrateur|Elle remet la petite roue.
-narrateur|Ça fait toc, tout doux.
-maman|Tu as mis le train ?
-enfant-f|Oui, maman.
-narrateur|Chouchou met ses chaussures.
-narrateur|Les lacets font un petit bruit.
-papa|On ouvre ?
-enfant-f|L'allée.
-narrateur|Maman ouvre la porte.
-narrateur|L'air sent la terre mouillée.
-narrateur|Les dalles commencent à être tièdes.
-narrateur|Chouchou sort le train.
-narrateur|Elle le pose sur une dalle.
+          <t>papa|Il va jusqu'à la dernière dalle ?
+enfant-f|Oui, papa.
+narrateur|Une feuille mouillée barre une dalle.
+narrateur|Le wagon s'arrête contre le bord.
+enfant-f|Je le porte !
+narrateur|Elle saisit le train trop vite.
+narrateur|Une roue quitte la dalle.
+enfant-f|Oh.
+narrateur|Chouchou s'arrête.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Elle refuse de foncer.
+narrateur|Le train revient sur la dalle sèche.
+narrateur|Elle écarte la feuille du bout des doigts.
+narrateur|La dalle est libre, un peu sombre.
 enfant-f|Roule.
 narrateur|Le wagon avance.
 narrateur|Toc.
 narrateur|Une autre dalle, plus loin.
-papa|Il va jusqu'au merle.
-maman|Une chose, puis la suivante.
-maman|Et le train est parti.
-narrateur|Le merle penche la tête.
-enfant-f|Il me regarde.</t>
+narrateur|L'éclat de wagon tremble, puis tient.
+papa|Il a passé la feuille.
+maman|La dernière dalle est près du portail.
+enfant-f|J'y vais.
+narrateur|Chouchou marche à côté, sans le porter.
+narrateur|Le bois continue son petit bruit.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>porte</t>
+          <t>porte,feuille</t>
         </is>
       </c>
     </row>
@@ -1959,17 +2007,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le toit est rouge au soleil. Il a fait tout le chemin. Toi aussi. Le merle chante encore, tout au fond. Le wagon est chaud, sous tes doigts. Les dalles sont chaudes maintenant.</t>
+          <t>Ils s'arrêtent près du portail. Le toit est rouge au soleil. Il a fait tout le chemin. Toi aussi. Le wagon est chaud, sous ses doigts. Les dalles sont chaudes maintenant. Tu sens le bois ? Oui, maman. Chouchou glisse le train sans se presser. Le bois repose contre sa hanche. Comme sur le rebord, papa ! Tu le vois, toi ? Oui, sur le toit rouge. On est bien, ici. La terre mouillée reste dans l'air. L'éclat de wagon tient sur le toit.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le toit est rouge au soleil. Il a fait tout le chemin. Toi aussi. Le merle chante encore, tout au fond. Le wagon est chaud, sous tes doigts. Les dalles sont chaudes maintenant.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils s'arrêtent près du portail. Le toit est rouge au soleil. Il a fait tout le chemin. Toi aussi. Le wagon est chaud, sous ses doigts. Les dalles sont chaudes maintenant. Tu sens le bois ? Oui, maman. Chouchou glisse le train sans se presser. Le bois repose contre sa hanche. Comme sur le rebord, papa ! Tu le vois, toi ? Oui, sur le toit rouge. On est bien, ici. La terre mouillée reste dans l'air. L'&lt;emphasis level="moderate"&gt;éclat de wagon&lt;/emphasis&gt; tient sur le toit.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils s'arrêtent près du portail. Le toit est rouge au soleil. Il a fait tout le chemin. Toi aussi. Le wagon est chaud, sous ses doigts. Les dalles sont chaudes maintenant. Tu sens le bois ? Oui, maman. Chouchou glisse le train sans se presser. Le bois repose contre sa hanche. Comme sur le rebord, papa ! Tu le vois, toi ? Oui, sur le toit rouge. On est bien, ici. La terre mouillée reste dans l'air. L'&lt;emphasis&gt;éclat de wagon&lt;/emphasis&gt; tient sur le toit.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2016,18 +2064,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2036,12 +2084,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2050,17 +2098,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de wagon</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2069,11 +2121,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2082,29 +2134,48 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_toit; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-f|Le toit est rouge au soleil.
-papa|Il a fait tout le chemin.
-maman|Toi aussi.
-narrateur|Le merle chante encore, tout au fond.
-papa|Le wagon est chaud, sous tes doigts.
-narrateur|Les dalles sont chaudes maintenant.</t>
+          <t>narrateur|Ils s'arrêtent près du portail.
+narrateur|Le toit est rouge au soleil.
+enfant-f|Il a fait tout le chemin.
+papa|Toi aussi.
+narrateur|Le wagon est chaud, sous ses doigts.
+narrateur|Les dalles sont chaudes maintenant.
+maman|Tu sens le bois ?
+enfant-f|Oui, maman.
+narrateur|Chouchou glisse le train sans se presser.
+narrateur|Le bois repose contre sa hanche.
+enfant-f|Comme sur le rebord, papa !
+papa|Tu le vois, toi ?
+enfant-f|Oui, sur le toit rouge.
+maman|On est bien, ici.
+narrateur|La terre mouillée reste dans l'air.
+narrateur|L'éclat de wagon tient sur le toit.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>portail</t>
         </is>
       </c>
     </row>
@@ -2125,7 +2196,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2224,6 +2295,13 @@
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>